<commit_message>
Detect titles, multiple tables and footnotes in sheets; parse more number formats; support OR in query_table
- split_tables finds tables in a sheet: title rows, several tables
  separated by empty rows, empty rows inside a table, footnotes and
  tables that do not start in column A.
- parse_number handles English/German grouping, currency, percent,
  Norwegian ',-' and typographic minus.
- query_table conditions can contain alternatives separated by ' OR '.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/budsjett.xlsx
+++ b/samples/budsjett.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaksjoner" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tomt" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hjelpetall" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartal" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5113,4 +5114,151 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Kvartalsrapport 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Budsjett Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Avdeling</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Q1 budsjett</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Salg</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Faktisk Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Avdeling</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Q1 faktisk</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Salg</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1,250,000.50</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Over plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1.180.000,00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Serverkjøp</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>kr 95 000,-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kilde: regnskapssystemet, hentet 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>